<commit_message>
Publisher watermark on the files themselves; credit the publisher
- The watermark is now part of the content: drawn into PDF pages and images,
  tiled over each Word page, slide, sheet, e-book view and video. The
  full-screen overlay is gone.
- The admin chooses what it says (Restrictions: publisher name + second line,
  with a live preview). The name starts as the admin's name (migration 7) and
  is also shown as "Published by" on the file page, preview and reader.
- Sample files and covers credit the publisher instead of made-up authors;
  make-samples.mjs and make_demo_catalog.py take the publisher name.
</commit_message>
<xml_diff>
--- a/supabase/sample/files/lab-values-cheat-sheet.xlsx
+++ b/supabase/sample/files/lab-values-cheat-sheet.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -503,9 +503,14 @@
         <v>mg/dL</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Published by Fritz Rjhay Dela Cruz</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>